<commit_message>
Alteração de ficheiros acerca das us21/25
</commit_message>
<xml_diff>
--- a/docs/sprintC/PI-2023-24 Self-Assessment - SPRINT C.xlsx
+++ b/docs/sprintC/PI-2023-24 Self-Assessment - SPRINT C.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Francisco\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Me\Desktop\Projeto Final\lei-24-s2-1dp-g163\docs\sprintC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64796845-09D8-463E-B2D7-EE2D02873BA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{286360EE-990D-4383-85F5-D35040A1E1B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Group and Self Assessment" sheetId="2" r:id="rId1"/>
@@ -1856,33 +1856,33 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:T36"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="5.59765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="19" width="7.8984375" customWidth="1"/>
+    <col min="4" max="19" width="7.875" customWidth="1"/>
     <col min="20" max="20" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="21" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:20" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="24" t="s">
         <v>141</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="34" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
@@ -1891,13 +1891,13 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:20" ht="16.2" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="8" spans="1:20" ht="15.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="8" spans="1:20" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="E8" s="65" t="s">
@@ -1919,7 +1919,7 @@
       <c r="S8" s="66"/>
       <c r="T8" s="67"/>
     </row>
-    <row r="9" spans="1:20" ht="105.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:20" ht="105.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="42">
@@ -1986,7 +1986,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:20" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="62" t="s">
         <v>6</v>
       </c>
@@ -2025,7 +2025,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:20" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="63"/>
       <c r="C11" s="8" t="s">
         <v>7</v>
@@ -2050,7 +2050,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="12" spans="1:20" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="63"/>
       <c r="C12" s="8" t="s">
         <v>8</v>
@@ -2075,7 +2075,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="13" spans="1:20" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="63"/>
       <c r="C13" s="8" t="s">
         <v>9</v>
@@ -2100,7 +2100,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="14" spans="1:20" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="63"/>
       <c r="C14" s="8" t="s">
         <v>10</v>
@@ -2125,7 +2125,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="15" spans="1:20" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="63"/>
       <c r="C15" s="8" t="s">
         <v>11</v>
@@ -2150,7 +2150,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="16" spans="1:20" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="63"/>
       <c r="C16" s="8" t="s">
         <v>12</v>
@@ -2175,7 +2175,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="17" spans="1:19" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="63"/>
       <c r="C17" s="8" t="s">
         <v>13</v>
@@ -2200,7 +2200,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="18" spans="1:19" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B18" s="63"/>
       <c r="C18" s="8" t="s">
         <v>14</v>
@@ -2225,7 +2225,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="19" spans="1:19" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="63"/>
       <c r="C19" s="8" t="s">
         <v>15</v>
@@ -2250,7 +2250,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="20" spans="1:19" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B20" s="63"/>
       <c r="C20" s="8" t="s">
         <v>16</v>
@@ -2275,7 +2275,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="21" spans="1:19" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="63"/>
       <c r="C21" s="8" t="s">
         <v>17</v>
@@ -2300,7 +2300,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="22" spans="1:19" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B22" s="63"/>
       <c r="C22" s="8" t="s">
         <v>18</v>
@@ -2325,7 +2325,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="23" spans="1:19" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B23" s="63"/>
       <c r="C23" s="8" t="s">
         <v>19</v>
@@ -2350,7 +2350,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="24" spans="1:19" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B24" s="64"/>
       <c r="C24" s="40" t="s">
         <v>20</v>
@@ -2375,7 +2375,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="25" spans="1:19" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B25" s="1"/>
       <c r="C25" s="45" t="s">
         <v>5</v>
@@ -2442,27 +2442,27 @@
       </c>
       <c r="S25" s="53"/>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>0</v>
       </c>
@@ -2470,7 +2470,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>1</v>
       </c>
@@ -2478,7 +2478,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>2</v>
       </c>
@@ -2486,7 +2486,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>3</v>
       </c>
@@ -2494,7 +2494,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>4</v>
       </c>
@@ -2502,7 +2502,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>5</v>
       </c>
@@ -2529,21 +2529,21 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:J25"/>
-  <sheetFormatPr defaultColWidth="20.09765625" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="20.125" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.09765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="22.5" customWidth="1"/>
     <col min="5" max="10" width="27.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="30" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="62" t="s">
         <v>32</v>
       </c>
@@ -2575,7 +2575,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A4" s="63"/>
       <c r="B4" s="71"/>
       <c r="C4" s="71"/>
@@ -2599,7 +2599,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" ht="48" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="63"/>
       <c r="B5" s="71"/>
       <c r="C5" s="71"/>
@@ -2623,7 +2623,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>151</v>
       </c>
@@ -2649,7 +2649,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>152</v>
       </c>
@@ -2679,7 +2679,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>153</v>
       </c>
@@ -2707,7 +2707,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>154</v>
       </c>
@@ -2733,7 +2733,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>155</v>
       </c>
@@ -2759,7 +2759,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>142</v>
       </c>
@@ -2787,7 +2787,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>143</v>
       </c>
@@ -2815,7 +2815,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>144</v>
       </c>
@@ -2847,7 +2847,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
         <v>145</v>
       </c>
@@ -2877,7 +2877,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>146</v>
       </c>
@@ -2907,7 +2907,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
         <v>147</v>
       </c>
@@ -2937,7 +2937,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>148</v>
       </c>
@@ -2969,7 +2969,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
         <v>149</v>
       </c>
@@ -2997,7 +2997,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
         <v>156</v>
       </c>
@@ -3025,7 +3025,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
         <v>150</v>
       </c>
@@ -3053,7 +3053,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
         <v>161</v>
       </c>
@@ -3079,7 +3079,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" ht="63" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
         <v>162</v>
       </c>
@@ -3107,7 +3107,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A23" s="14"/>
       <c r="B23" s="29"/>
       <c r="C23" s="29"/>
@@ -3133,7 +3133,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A24" s="14"/>
       <c r="B24" s="29"/>
       <c r="C24" s="29"/>
@@ -3159,7 +3159,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" ht="48" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="22"/>
       <c r="B25" s="54"/>
       <c r="C25" s="54"/>
@@ -3225,24 +3225,24 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:Z10"/>
-  <sheetFormatPr defaultColWidth="10.8984375" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.8984375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="7.09765625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="17" width="5.59765625" style="1" customWidth="1"/>
-    <col min="18" max="18" width="12.09765625" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="20" width="16.3984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="7.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="17" width="5.625" style="1" customWidth="1"/>
+    <col min="18" max="18" width="12.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="20" width="16.375" style="1" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="17.5" style="1" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="17" style="1" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="16.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="16.3984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="16.375" style="1" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="11" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="8.3984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="28" width="7.3984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="16384" width="10.8984375" style="1"/>
+    <col min="26" max="26" width="8.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="28" width="7.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="29" max="16384" width="10.875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="21" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:26" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="24" t="s">
         <v>51</v>
       </c>
@@ -3261,8 +3261,8 @@
       <c r="N1" s="13"/>
       <c r="O1" s="13"/>
     </row>
-    <row r="2" spans="1:26" ht="16.2" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="3" spans="1:26" ht="57" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:26" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:26" ht="57" x14ac:dyDescent="0.25">
       <c r="A3" s="19" t="s">
         <v>52</v>
       </c>
@@ -3363,7 +3363,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:26" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:26" ht="63" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
         <v>54</v>
       </c>
@@ -3412,7 +3412,7 @@
       <c r="Y4" s="7"/>
       <c r="Z4" s="15"/>
     </row>
-    <row r="5" spans="1:26" ht="124.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:26" ht="110.25" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>61</v>
       </c>
@@ -3461,7 +3461,7 @@
       <c r="Y5" s="7"/>
       <c r="Z5" s="15"/>
     </row>
-    <row r="6" spans="1:26" ht="78" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:26" ht="78.75" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>68</v>
       </c>
@@ -3510,7 +3510,7 @@
       <c r="Y6" s="7"/>
       <c r="Z6" s="15"/>
     </row>
-    <row r="7" spans="1:26" ht="93.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:26" ht="78.75" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>74</v>
       </c>
@@ -3559,7 +3559,7 @@
       <c r="Y7" s="7"/>
       <c r="Z7" s="15"/>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>50</v>
       </c>
@@ -3637,7 +3637,7 @@
       <c r="Y8" s="7"/>
       <c r="Z8" s="15"/>
     </row>
-    <row r="9" spans="1:26" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:26" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
         <v>80</v>
       </c>
@@ -3712,7 +3712,7 @@
       <c r="Y9" s="23"/>
       <c r="Z9" s="16"/>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A10" s="5"/>
     </row>
   </sheetData>
@@ -3730,22 +3730,22 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:Z17"/>
-  <sheetFormatPr defaultColWidth="10.8984375" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.8984375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="7.09765625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="17" width="5.59765625" style="1" customWidth="1"/>
-    <col min="18" max="18" width="12.09765625" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="20" width="16.3984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="7.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="17" width="5.625" style="1" customWidth="1"/>
+    <col min="18" max="18" width="12.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="20" width="16.375" style="1" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="17.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="24" width="20.59765625" style="1" customWidth="1"/>
+    <col min="22" max="24" width="20.625" style="1" customWidth="1"/>
     <col min="25" max="25" width="11" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="8.3984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="28" width="7.3984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="16384" width="10.8984375" style="1"/>
+    <col min="26" max="26" width="8.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="28" width="7.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="29" max="16384" width="10.875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="21" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:26" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="24" t="s">
         <v>81</v>
       </c>
@@ -3764,7 +3764,7 @@
       <c r="N1" s="13"/>
       <c r="O1" s="13"/>
     </row>
-    <row r="3" spans="1:26" ht="57" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:26" ht="57" x14ac:dyDescent="0.25">
       <c r="A3" s="19" t="s">
         <v>52</v>
       </c>
@@ -3775,9 +3775,8 @@
         <f>'Group and Self Assessment'!C10</f>
         <v>1230684</v>
       </c>
-      <c r="D3" s="20" t="str">
-        <f>'Group and Self Assessment'!C11</f>
-        <v>Student 2</v>
+      <c r="D3" s="20">
+        <v>1210527</v>
       </c>
       <c r="E3" s="20" t="str">
         <f>'Group and Self Assessment'!C12</f>
@@ -3865,7 +3864,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:26" ht="144.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:26" ht="144.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
         <v>82</v>
       </c>
@@ -3875,7 +3874,9 @@
       <c r="C4" s="25">
         <v>5</v>
       </c>
-      <c r="D4" s="25"/>
+      <c r="D4" s="25">
+        <v>0</v>
+      </c>
       <c r="E4" s="25"/>
       <c r="F4" s="25"/>
       <c r="G4" s="25"/>
@@ -3891,7 +3892,7 @@
       <c r="Q4" s="25"/>
       <c r="R4" s="55">
         <f t="shared" ref="R4:R7" si="0">AVERAGE(C4:Q4)</f>
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="S4" s="59" t="s">
         <v>83</v>
@@ -3914,7 +3915,7 @@
       <c r="Y4" s="56"/>
       <c r="Z4" s="15"/>
     </row>
-    <row r="5" spans="1:26" ht="101.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:26" ht="101.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>89</v>
       </c>
@@ -3924,7 +3925,9 @@
       <c r="C5" s="25">
         <v>5</v>
       </c>
-      <c r="D5" s="25"/>
+      <c r="D5" s="25">
+        <v>5</v>
+      </c>
       <c r="E5" s="25"/>
       <c r="F5" s="25"/>
       <c r="G5" s="25"/>
@@ -3963,7 +3966,7 @@
       <c r="Y5" s="56"/>
       <c r="Z5" s="15"/>
     </row>
-    <row r="6" spans="1:26" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:26" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>96</v>
       </c>
@@ -3973,7 +3976,9 @@
       <c r="C6" s="25">
         <v>5</v>
       </c>
-      <c r="D6" s="25"/>
+      <c r="D6" s="25">
+        <v>5</v>
+      </c>
       <c r="E6" s="25"/>
       <c r="F6" s="25"/>
       <c r="G6" s="25"/>
@@ -4012,7 +4017,7 @@
       <c r="Y6" s="56"/>
       <c r="Z6" s="15"/>
     </row>
-    <row r="7" spans="1:26" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:26" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>103</v>
       </c>
@@ -4022,7 +4027,9 @@
       <c r="C7" s="25">
         <v>5</v>
       </c>
-      <c r="D7" s="25"/>
+      <c r="D7" s="25">
+        <v>5</v>
+      </c>
       <c r="E7" s="25"/>
       <c r="F7" s="25"/>
       <c r="G7" s="25"/>
@@ -4061,7 +4068,7 @@
       <c r="Y7" s="56"/>
       <c r="Z7" s="15"/>
     </row>
-    <row r="8" spans="1:26" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:26" ht="63" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>109</v>
       </c>
@@ -4071,7 +4078,9 @@
       <c r="C8" s="25">
         <v>5</v>
       </c>
-      <c r="D8" s="25"/>
+      <c r="D8" s="25">
+        <v>3</v>
+      </c>
       <c r="E8" s="25"/>
       <c r="F8" s="25"/>
       <c r="G8" s="25"/>
@@ -4087,7 +4096,7 @@
       <c r="Q8" s="25"/>
       <c r="R8" s="55">
         <f t="shared" ref="R8:R12" si="1">AVERAGE(C8:Q8)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S8" s="59" t="s">
         <v>97</v>
@@ -4110,7 +4119,7 @@
       <c r="Y8" s="56"/>
       <c r="Z8" s="15"/>
     </row>
-    <row r="9" spans="1:26" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:26" ht="63" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>115</v>
       </c>
@@ -4120,7 +4129,9 @@
       <c r="C9" s="25">
         <v>5</v>
       </c>
-      <c r="D9" s="25"/>
+      <c r="D9" s="25">
+        <v>3</v>
+      </c>
       <c r="E9" s="25"/>
       <c r="F9" s="25"/>
       <c r="G9" s="25"/>
@@ -4136,7 +4147,7 @@
       <c r="Q9" s="25"/>
       <c r="R9" s="55">
         <f t="shared" ref="R9:R11" si="2">AVERAGE(C9:Q9)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S9" s="59" t="s">
         <v>116</v>
@@ -4155,7 +4166,7 @@
       <c r="Y9" s="56"/>
       <c r="Z9" s="15"/>
     </row>
-    <row r="10" spans="1:26" ht="93.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:26" ht="78.75" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>120</v>
       </c>
@@ -4165,7 +4176,9 @@
       <c r="C10" s="25">
         <v>5</v>
       </c>
-      <c r="D10" s="25"/>
+      <c r="D10" s="25">
+        <v>0</v>
+      </c>
       <c r="E10" s="25"/>
       <c r="F10" s="25"/>
       <c r="G10" s="25"/>
@@ -4181,7 +4194,7 @@
       <c r="Q10" s="25"/>
       <c r="R10" s="55">
         <f t="shared" si="2"/>
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="S10" s="59" t="s">
         <v>116</v>
@@ -4204,7 +4217,7 @@
       <c r="Y10" s="56"/>
       <c r="Z10" s="15"/>
     </row>
-    <row r="11" spans="1:26" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:26" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>126</v>
       </c>
@@ -4214,7 +4227,9 @@
       <c r="C11" s="25">
         <v>5</v>
       </c>
-      <c r="D11" s="25"/>
+      <c r="D11" s="25">
+        <v>0</v>
+      </c>
       <c r="E11" s="25"/>
       <c r="F11" s="25"/>
       <c r="G11" s="25"/>
@@ -4230,7 +4245,7 @@
       <c r="Q11" s="25"/>
       <c r="R11" s="55">
         <f t="shared" si="2"/>
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="S11" s="59" t="s">
         <v>116</v>
@@ -4253,7 +4268,7 @@
       <c r="Y11" s="56"/>
       <c r="Z11" s="15"/>
     </row>
-    <row r="12" spans="1:26" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:26" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>132</v>
       </c>
@@ -4263,7 +4278,9 @@
       <c r="C12" s="25">
         <v>5</v>
       </c>
-      <c r="D12" s="25"/>
+      <c r="D12" s="25">
+        <v>0</v>
+      </c>
       <c r="E12" s="25"/>
       <c r="F12" s="25"/>
       <c r="G12" s="25"/>
@@ -4279,7 +4296,7 @@
       <c r="Q12" s="25"/>
       <c r="R12" s="55">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="S12" s="59" t="s">
         <v>116</v>
@@ -4302,7 +4319,7 @@
       <c r="Y12" s="56"/>
       <c r="Z12" s="15"/>
     </row>
-    <row r="13" spans="1:26" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:26" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>133</v>
       </c>
@@ -4312,7 +4329,9 @@
       <c r="C13" s="25">
         <v>5</v>
       </c>
-      <c r="D13" s="25"/>
+      <c r="D13" s="25">
+        <v>5</v>
+      </c>
       <c r="E13" s="25"/>
       <c r="F13" s="25"/>
       <c r="G13" s="25"/>
@@ -4351,7 +4370,7 @@
       <c r="Y13" s="56"/>
       <c r="Z13" s="15"/>
     </row>
-    <row r="14" spans="1:26" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:26" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
         <v>140</v>
       </c>
@@ -4361,7 +4380,9 @@
       <c r="C14" s="25">
         <v>5</v>
       </c>
-      <c r="D14" s="25"/>
+      <c r="D14" s="25">
+        <v>5</v>
+      </c>
       <c r="E14" s="25"/>
       <c r="F14" s="25"/>
       <c r="G14" s="25"/>
@@ -4400,7 +4421,7 @@
       <c r="Y14" s="56"/>
       <c r="Z14" s="15"/>
     </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>50</v>
       </c>
@@ -4414,7 +4435,7 @@
       </c>
       <c r="D15" s="7">
         <f t="shared" ref="D15:Q15" si="4">SUMPRODUCT(D4:D14,$B$4:$B$14)</f>
-        <v>0</v>
+        <v>2.7</v>
       </c>
       <c r="E15" s="7">
         <f t="shared" si="4"/>
@@ -4478,7 +4499,7 @@
       <c r="Y15" s="7"/>
       <c r="Z15" s="15"/>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16" s="22" t="s">
         <v>80</v>
       </c>
@@ -4489,7 +4510,7 @@
       </c>
       <c r="D16" s="23">
         <f t="shared" ref="D16:Q16" si="5">D15/5*20</f>
-        <v>0</v>
+        <v>10.8</v>
       </c>
       <c r="E16" s="23">
         <f t="shared" si="5"/>
@@ -4553,7 +4574,7 @@
       <c r="Y16" s="23"/>
       <c r="Z16" s="16"/>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="5"/>
     </row>
   </sheetData>
@@ -4568,6 +4589,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005836243B3C47804EAF5FFDD9F066FCC7" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9d21ddf3f0b128e39c9d770c8c903166">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b0326308c339679ad994635f2c691325" ns2:_="">
     <xsd:import namespace="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
@@ -4751,22 +4787,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D8D82CB-2E6F-4A14-B6B4-DFDD1BBD70FC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F61419B8-A98A-41CD-95EE-48A4F975B8D1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23B77F7C-EE47-4FBD-B078-6536C1487A1E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4782,28 +4827,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F61419B8-A98A-41CD-95EE-48A4F975B8D1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D8D82CB-2E6F-4A14-B6B4-DFDD1BBD70FC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
US028: Atualização do design
</commit_message>
<xml_diff>
--- a/docs/sprintC/PI-2023-24 Self-Assessment - SPRINT C.xlsx
+++ b/docs/sprintC/PI-2023-24 Self-Assessment - SPRINT C.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10512"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Me\Desktop\Projeto Final\lei-24-s2-1dp-g163\docs\sprintC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/inesgomesoliveira/Desktop/lei-24-s2-1dp-g163/docs/sprintC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{286360EE-990D-4383-85F5-D35040A1E1B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB5A2AD4-23AF-0B4F-9BA2-8DD0DEE1D2A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Group and Self Assessment" sheetId="2" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="168">
   <si>
     <t>Fill the cells with a blue background</t>
   </si>
@@ -66,9 +66,6 @@
   </si>
   <si>
     <t>List A</t>
-  </si>
-  <si>
-    <t>Student 2</t>
   </si>
   <si>
     <t>Student 3</t>
@@ -1856,33 +1853,33 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:T36"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="5.625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="19" width="7.875" customWidth="1"/>
+    <col min="4" max="19" width="7.83203125" customWidth="1"/>
     <col min="20" max="20" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" ht="21" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A2" s="34" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" ht="17" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
@@ -1891,13 +1888,13 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="8" spans="1:20" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:20" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="1:20" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="E8" s="65" t="s">
@@ -1919,16 +1916,16 @@
       <c r="S8" s="66"/>
       <c r="T8" s="67"/>
     </row>
-    <row r="9" spans="1:20" ht="105.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:20" ht="106" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="42">
         <f>C10</f>
         <v>1230684</v>
       </c>
-      <c r="E9" s="43" t="str">
+      <c r="E9" s="43">
         <f>C11</f>
-        <v>Student 2</v>
+        <v>1231205</v>
       </c>
       <c r="F9" s="43" t="str">
         <f>C12</f>
@@ -1986,7 +1983,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:20" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B10" s="62" t="s">
         <v>6</v>
       </c>
@@ -2025,13 +2022,17 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:20" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B11" s="63"/>
-      <c r="C11" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D11" s="9"/>
-      <c r="E11" s="36"/>
+      <c r="C11" s="8">
+        <v>1231205</v>
+      </c>
+      <c r="D11" s="9">
+        <v>5</v>
+      </c>
+      <c r="E11" s="36">
+        <v>4</v>
+      </c>
       <c r="F11" s="35"/>
       <c r="G11" s="8"/>
       <c r="H11" s="8"/>
@@ -2045,15 +2046,15 @@
       <c r="P11" s="8"/>
       <c r="Q11" s="8"/>
       <c r="R11" s="10"/>
-      <c r="S11" s="51" t="e">
+      <c r="S11" s="51">
         <f t="shared" ref="S11:S24" si="0">AVERAGE(D11:R11)</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="12" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B12" s="63"/>
       <c r="C12" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D12" s="8"/>
       <c r="E12" s="9"/>
@@ -2075,10 +2076,10 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="13" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:20" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B13" s="63"/>
       <c r="C13" s="8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D13" s="8"/>
       <c r="E13" s="8"/>
@@ -2100,10 +2101,10 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="14" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:20" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B14" s="63"/>
       <c r="C14" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D14" s="8"/>
       <c r="E14" s="8"/>
@@ -2125,10 +2126,10 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="15" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:20" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B15" s="63"/>
       <c r="C15" s="8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D15" s="8"/>
       <c r="E15" s="8"/>
@@ -2150,10 +2151,10 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="16" spans="1:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:20" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B16" s="63"/>
       <c r="C16" s="8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
@@ -2175,10 +2176,10 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="17" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:19" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B17" s="63"/>
       <c r="C17" s="8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D17" s="8"/>
       <c r="E17" s="8"/>
@@ -2200,10 +2201,10 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="18" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:19" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B18" s="63"/>
       <c r="C18" s="8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D18" s="8"/>
       <c r="E18" s="8"/>
@@ -2225,10 +2226,10 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="19" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:19" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B19" s="63"/>
       <c r="C19" s="8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D19" s="8"/>
       <c r="E19" s="8"/>
@@ -2250,10 +2251,10 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="20" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:19" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B20" s="63"/>
       <c r="C20" s="8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D20" s="8"/>
       <c r="E20" s="8"/>
@@ -2275,10 +2276,10 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="21" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:19" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B21" s="63"/>
       <c r="C21" s="8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D21" s="8"/>
       <c r="E21" s="8"/>
@@ -2300,10 +2301,10 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="22" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:19" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B22" s="63"/>
       <c r="C22" s="8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D22" s="8"/>
       <c r="E22" s="8"/>
@@ -2325,10 +2326,10 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="23" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:19" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B23" s="63"/>
       <c r="C23" s="8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D23" s="8"/>
       <c r="E23" s="8"/>
@@ -2350,10 +2351,10 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="24" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:19" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B24" s="64"/>
       <c r="C24" s="40" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D24" s="40"/>
       <c r="E24" s="40"/>
@@ -2375,7 +2376,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="25" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:19" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B25" s="1"/>
       <c r="C25" s="45" t="s">
         <v>5</v>
@@ -2386,7 +2387,7 @@
       </c>
       <c r="E25" s="46">
         <f t="shared" ref="E25:R25" si="1">AVERAGE(E10:E24)</f>
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="F25" s="46">
         <f t="shared" si="1"/>
@@ -2442,72 +2443,72 @@
       </c>
       <c r="S25" s="53"/>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="28" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+    <row r="29" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A29" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
+    <row r="30" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+    <row r="31" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A31">
+        <v>0</v>
+      </c>
+      <c r="B31" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A31">
-        <v>0</v>
-      </c>
-      <c r="B31" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>1</v>
       </c>
       <c r="B32" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>2</v>
       </c>
       <c r="B33" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>3</v>
       </c>
       <c r="B34" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>4</v>
       </c>
       <c r="B35" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>5</v>
       </c>
       <c r="B36" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -2529,32 +2530,32 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:J25"/>
-  <sheetFormatPr defaultColWidth="20.125" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="20.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="22.5" customWidth="1"/>
     <col min="5" max="10" width="27.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="30" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3" s="62" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="62" t="s">
+      <c r="B3" s="70" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="70" t="s">
+      <c r="C3" s="70" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="70" t="s">
+      <c r="D3" s="68" t="s">
         <v>34</v>
-      </c>
-      <c r="D3" s="68" t="s">
-        <v>35</v>
       </c>
       <c r="E3" s="11">
         <v>0</v>
@@ -2575,249 +2576,253 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A4" s="63"/>
       <c r="B4" s="71"/>
       <c r="C4" s="71"/>
       <c r="D4" s="69"/>
       <c r="E4" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="F4" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="G4" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="H4" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="I4" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="I4" s="7" t="s">
+      <c r="J4" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="J4" s="15" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="48" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:10" ht="52" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="63"/>
       <c r="B5" s="71"/>
       <c r="C5" s="71"/>
       <c r="D5" s="69"/>
       <c r="E5" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="F5" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="F5" s="23" t="s">
+      <c r="G5" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="G5" s="23" t="s">
+      <c r="H5" s="23" t="s">
         <v>44</v>
       </c>
-      <c r="H5" s="23" t="s">
+      <c r="I5" s="23" t="s">
         <v>45</v>
       </c>
-      <c r="I5" s="23" t="s">
+      <c r="J5" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="J5" s="16" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A6" s="14" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B6" s="29"/>
       <c r="C6" s="29"/>
       <c r="D6" s="60"/>
       <c r="E6" s="31" t="s">
+        <v>41</v>
+      </c>
+      <c r="F6" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="F6" s="32" t="s">
+      <c r="G6" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="G6" s="32" t="s">
+      <c r="H6" s="32" t="s">
         <v>44</v>
       </c>
-      <c r="H6" s="32" t="s">
+      <c r="I6" s="32" t="s">
         <v>45</v>
       </c>
-      <c r="I6" s="32" t="s">
-        <v>46</v>
-      </c>
       <c r="J6" s="33" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A7" s="14" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B7" s="29">
         <v>1230684</v>
       </c>
       <c r="C7" s="29"/>
       <c r="D7" s="60" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E7" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="F7" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="G7" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="H7" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="I7" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="I7" s="7" t="s">
-        <v>46</v>
-      </c>
       <c r="J7" s="33" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A8" s="14" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B8" s="60" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C8" s="29"/>
       <c r="D8" s="60"/>
       <c r="E8" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="F8" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="G8" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="H8" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="I8" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="I8" s="7" t="s">
-        <v>46</v>
-      </c>
       <c r="J8" s="33" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A9" s="14" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B9" s="29"/>
       <c r="C9" s="29"/>
       <c r="D9" s="60"/>
       <c r="E9" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="F9" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="G9" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="H9" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="H9" s="7" t="s">
+      <c r="I9" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="I9" s="7" t="s">
-        <v>46</v>
-      </c>
       <c r="J9" s="33" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A10" s="14" t="s">
-        <v>155</v>
-      </c>
-      <c r="B10" s="29"/>
+        <v>154</v>
+      </c>
+      <c r="B10" s="29">
+        <v>1231205</v>
+      </c>
       <c r="C10" s="29"/>
       <c r="D10" s="60"/>
       <c r="E10" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="F10" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="G10" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="H10" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="H10" s="7" t="s">
+      <c r="I10" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="I10" s="7" t="s">
-        <v>46</v>
-      </c>
       <c r="J10" s="33" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A11" s="14" t="s">
-        <v>142</v>
-      </c>
-      <c r="B11" s="29"/>
+        <v>141</v>
+      </c>
+      <c r="B11" s="29">
+        <v>1231205</v>
+      </c>
       <c r="C11" s="29"/>
       <c r="D11" s="60" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E11" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="F11" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="G11" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G11" s="7" t="s">
+      <c r="H11" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="H11" s="7" t="s">
+      <c r="I11" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="I11" s="7" t="s">
-        <v>46</v>
-      </c>
       <c r="J11" s="33" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A12" s="14" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B12" s="29"/>
       <c r="C12" s="29"/>
       <c r="D12" s="60" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E12" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="F12" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="G12" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="H12" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="H12" s="7" t="s">
+      <c r="I12" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="I12" s="7" t="s">
-        <v>46</v>
-      </c>
       <c r="J12" s="33" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A13" s="14" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B13" s="29">
         <v>1230684</v>
@@ -2826,120 +2831,122 @@
         <v>5</v>
       </c>
       <c r="D13" s="60" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E13" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="F13" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="G13" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G13" s="7" t="s">
+      <c r="H13" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="H13" s="7" t="s">
+      <c r="I13" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="I13" s="7" t="s">
-        <v>46</v>
-      </c>
       <c r="J13" s="33" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A14" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B14" s="29"/>
       <c r="C14" s="29">
         <v>5</v>
       </c>
       <c r="D14" s="60" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E14" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="F14" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="G14" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G14" s="7" t="s">
+      <c r="H14" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="H14" s="7" t="s">
+      <c r="I14" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="I14" s="7" t="s">
-        <v>46</v>
-      </c>
       <c r="J14" s="33" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A15" s="14" t="s">
-        <v>146</v>
-      </c>
-      <c r="B15" s="29"/>
+        <v>145</v>
+      </c>
+      <c r="B15" s="29">
+        <v>1231205</v>
+      </c>
       <c r="C15" s="29">
         <v>5</v>
       </c>
       <c r="D15" s="60" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E15" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="F15" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="G15" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G15" s="7" t="s">
+      <c r="H15" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="H15" s="7" t="s">
+      <c r="I15" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="I15" s="7" t="s">
-        <v>46</v>
-      </c>
       <c r="J15" s="33" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A16" s="14" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B16" s="29"/>
       <c r="C16" s="29">
         <v>5</v>
       </c>
       <c r="D16" s="60" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E16" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="F16" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="G16" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G16" s="7" t="s">
+      <c r="H16" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="H16" s="7" t="s">
+      <c r="I16" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="I16" s="7" t="s">
-        <v>46</v>
-      </c>
       <c r="J16" s="33" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A17" s="14" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B17" s="29">
         <v>1230684</v>
@@ -2948,241 +2955,243 @@
         <v>5</v>
       </c>
       <c r="D17" s="60" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E17" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="F17" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="G17" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G17" s="7" t="s">
+      <c r="H17" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="H17" s="7" t="s">
+      <c r="I17" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="I17" s="7" t="s">
-        <v>46</v>
-      </c>
       <c r="J17" s="33" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A18" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B18" s="29"/>
       <c r="C18" s="29"/>
       <c r="D18" s="60" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E18" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="F18" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F18" s="7" t="s">
+      <c r="G18" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G18" s="7" t="s">
+      <c r="H18" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="H18" s="7" t="s">
+      <c r="I18" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="I18" s="7" t="s">
-        <v>46</v>
-      </c>
       <c r="J18" s="33" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A19" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="B19" s="29"/>
+        <v>155</v>
+      </c>
+      <c r="B19" s="29">
+        <v>1231205</v>
+      </c>
       <c r="C19" s="29"/>
       <c r="D19" s="60" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E19" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="F19" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F19" s="7" t="s">
+      <c r="G19" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G19" s="7" t="s">
+      <c r="H19" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="H19" s="7" t="s">
+      <c r="I19" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="I19" s="7" t="s">
-        <v>46</v>
-      </c>
       <c r="J19" s="33" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A20" s="14" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B20" s="29"/>
       <c r="C20" s="29"/>
       <c r="D20" s="60" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E20" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="F20" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F20" s="7" t="s">
+      <c r="G20" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G20" s="7" t="s">
+      <c r="H20" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="H20" s="7" t="s">
+      <c r="I20" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="I20" s="7" t="s">
-        <v>46</v>
-      </c>
       <c r="J20" s="33" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A21" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B21" s="29"/>
       <c r="C21" s="29"/>
       <c r="D21" s="60"/>
       <c r="E21" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="F21" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F21" s="7" t="s">
+      <c r="G21" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G21" s="7" t="s">
+      <c r="H21" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="H21" s="7" t="s">
+      <c r="I21" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="I21" s="7" t="s">
-        <v>46</v>
-      </c>
       <c r="J21" s="33" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="63" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="68" x14ac:dyDescent="0.2">
       <c r="A22" s="14" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B22" s="29"/>
       <c r="C22" s="29"/>
       <c r="D22" s="60" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E22" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="F22" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F22" s="7" t="s">
+      <c r="G22" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G22" s="7" t="s">
+      <c r="H22" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="H22" s="7" t="s">
+      <c r="I22" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="I22" s="7" t="s">
-        <v>46</v>
-      </c>
       <c r="J22" s="33" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A23" s="14"/>
       <c r="B23" s="29"/>
       <c r="C23" s="29"/>
       <c r="D23" s="60" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E23" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="F23" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F23" s="7" t="s">
+      <c r="G23" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G23" s="7" t="s">
+      <c r="H23" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="H23" s="7" t="s">
+      <c r="I23" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="I23" s="7" t="s">
-        <v>46</v>
-      </c>
       <c r="J23" s="33" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A24" s="14"/>
       <c r="B24" s="29"/>
       <c r="C24" s="29"/>
       <c r="D24" s="60" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E24" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="F24" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F24" s="7" t="s">
+      <c r="G24" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G24" s="7" t="s">
+      <c r="H24" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="H24" s="7" t="s">
+      <c r="I24" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="I24" s="7" t="s">
-        <v>46</v>
-      </c>
       <c r="J24" s="33" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" ht="48" thickBot="1" x14ac:dyDescent="0.3">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="52" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A25" s="22"/>
       <c r="B25" s="54"/>
       <c r="C25" s="54"/>
       <c r="D25" s="61" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E25" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="F25" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="F25" s="23" t="s">
+      <c r="G25" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="G25" s="23" t="s">
+      <c r="H25" s="23" t="s">
         <v>44</v>
       </c>
-      <c r="H25" s="23" t="s">
+      <c r="I25" s="23" t="s">
         <v>45</v>
       </c>
-      <c r="I25" s="23" t="s">
-        <v>46</v>
-      </c>
       <c r="J25" s="33" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -3225,26 +3234,26 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:Z10"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="7.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="17" width="5.625" style="1" customWidth="1"/>
-    <col min="18" max="18" width="12.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="20" width="16.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.83203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="7.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="17" width="5.6640625" style="1" customWidth="1"/>
+    <col min="18" max="18" width="12.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="20" width="16.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="17.5" style="1" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="17" style="1" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="16.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="16.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="16.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="11" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="8.375" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="28" width="7.375" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="16384" width="10.875" style="1"/>
+    <col min="26" max="26" width="8.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="28" width="7.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="29" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" ht="21" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B1" s="13"/>
       <c r="C1" s="13"/>
@@ -3261,21 +3270,21 @@
       <c r="N1" s="13"/>
       <c r="O1" s="13"/>
     </row>
-    <row r="2" spans="1:26" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:26" ht="57" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:26" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:26" ht="57" x14ac:dyDescent="0.2">
       <c r="A3" s="19" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C3" s="20">
         <f>'Group and Self Assessment'!C10</f>
         <v>1230684</v>
       </c>
-      <c r="D3" s="20" t="str">
+      <c r="D3" s="20">
         <f>'Group and Self Assessment'!C11</f>
-        <v>Student 2</v>
+        <v>1231205</v>
       </c>
       <c r="E3" s="20" t="str">
         <f>'Group and Self Assessment'!C12</f>
@@ -3357,15 +3366,15 @@
         <v>5</v>
       </c>
       <c r="Y3" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="Z3" s="12" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" ht="68" x14ac:dyDescent="0.2">
+      <c r="A4" s="14" t="s">
         <v>53</v>
-      </c>
-      <c r="Z3" s="12" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="4" spans="1:26" ht="63" x14ac:dyDescent="0.25">
-      <c r="A4" s="14" t="s">
-        <v>54</v>
       </c>
       <c r="B4" s="17">
         <v>0.1</v>
@@ -3373,7 +3382,9 @@
       <c r="C4" s="25">
         <v>4</v>
       </c>
-      <c r="D4" s="25"/>
+      <c r="D4" s="25">
+        <v>4</v>
+      </c>
       <c r="E4" s="25"/>
       <c r="F4" s="25"/>
       <c r="G4" s="25"/>
@@ -3392,29 +3403,29 @@
         <v>4</v>
       </c>
       <c r="S4" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="T4" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="T4" s="7" t="s">
+      <c r="U4" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="U4" s="7" t="s">
+      <c r="V4" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="V4" s="7" t="s">
+      <c r="W4" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="W4" s="7" t="s">
+      <c r="X4" s="7" t="s">
         <v>59</v>
-      </c>
-      <c r="X4" s="7" t="s">
-        <v>60</v>
       </c>
       <c r="Y4" s="7"/>
       <c r="Z4" s="15"/>
     </row>
-    <row r="5" spans="1:26" ht="110.25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:26" ht="119" x14ac:dyDescent="0.2">
       <c r="A5" s="14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B5" s="17">
         <v>0.2</v>
@@ -3422,7 +3433,9 @@
       <c r="C5" s="25">
         <v>4</v>
       </c>
-      <c r="D5" s="25"/>
+      <c r="D5" s="25">
+        <v>4</v>
+      </c>
       <c r="E5" s="25"/>
       <c r="F5" s="25"/>
       <c r="G5" s="25"/>
@@ -3441,29 +3454,29 @@
         <v>4</v>
       </c>
       <c r="S5" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="T5" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="T5" s="7" t="s">
+      <c r="U5" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="U5" s="7" t="s">
+      <c r="V5" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="V5" s="7" t="s">
+      <c r="W5" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="W5" s="7" t="s">
+      <c r="X5" s="7" t="s">
         <v>66</v>
-      </c>
-      <c r="X5" s="7" t="s">
-        <v>67</v>
       </c>
       <c r="Y5" s="7"/>
       <c r="Z5" s="15"/>
     </row>
-    <row r="6" spans="1:26" ht="78.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:26" ht="85" x14ac:dyDescent="0.2">
       <c r="A6" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B6" s="17">
         <v>0.5</v>
@@ -3471,7 +3484,9 @@
       <c r="C6" s="25">
         <v>5</v>
       </c>
-      <c r="D6" s="25"/>
+      <c r="D6" s="25">
+        <v>4</v>
+      </c>
       <c r="E6" s="25"/>
       <c r="F6" s="25"/>
       <c r="G6" s="25"/>
@@ -3487,32 +3502,32 @@
       <c r="Q6" s="25"/>
       <c r="R6" s="27">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="S6" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="T6" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="T6" s="7" t="s">
+      <c r="U6" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="U6" s="7" t="s">
+      <c r="V6" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="V6" s="7" t="s">
+      <c r="W6" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="W6" s="7" t="s">
-        <v>73</v>
-      </c>
       <c r="X6" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Y6" s="7"/>
       <c r="Z6" s="15"/>
     </row>
-    <row r="7" spans="1:26" ht="78.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:26" ht="102" x14ac:dyDescent="0.2">
       <c r="A7" s="14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B7" s="17">
         <v>0.2</v>
@@ -3520,7 +3535,9 @@
       <c r="C7" s="25">
         <v>5</v>
       </c>
-      <c r="D7" s="25"/>
+      <c r="D7" s="25">
+        <v>4</v>
+      </c>
       <c r="E7" s="25"/>
       <c r="F7" s="25"/>
       <c r="G7" s="25"/>
@@ -3536,32 +3553,32 @@
       <c r="Q7" s="25"/>
       <c r="R7" s="27">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="S7" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="T7" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="T7" s="7" t="s">
+      <c r="U7" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="U7" s="7" t="s">
+      <c r="V7" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="V7" s="7" t="s">
+      <c r="W7" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="W7" s="7" t="s">
-        <v>79</v>
-      </c>
       <c r="X7" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="Y7" s="7"/>
       <c r="Z7" s="15"/>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:26" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B8" s="18">
         <f>SUM(B4:B7)</f>
@@ -3573,7 +3590,7 @@
       </c>
       <c r="D8" s="7">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E8" s="7">
         <f t="shared" si="1"/>
@@ -3637,9 +3654,9 @@
       <c r="Y8" s="7"/>
       <c r="Z8" s="15"/>
     </row>
-    <row r="9" spans="1:26" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:26" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="22" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B9" s="23"/>
       <c r="C9" s="23">
@@ -3648,7 +3665,7 @@
       </c>
       <c r="D9" s="23">
         <f t="shared" ref="D9:Q9" si="2">D8/5*20</f>
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="E9" s="23">
         <f t="shared" si="2"/>
@@ -3712,7 +3729,7 @@
       <c r="Y9" s="23"/>
       <c r="Z9" s="16"/>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A10" s="5"/>
     </row>
   </sheetData>
@@ -3730,24 +3747,24 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:Z17"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="7.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="17" width="5.625" style="1" customWidth="1"/>
-    <col min="18" max="18" width="12.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="20" width="16.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.83203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="7.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="17" width="5.6640625" style="1" customWidth="1"/>
+    <col min="18" max="18" width="12.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="20" width="16.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="17.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="24" width="20.625" style="1" customWidth="1"/>
+    <col min="22" max="24" width="20.6640625" style="1" customWidth="1"/>
     <col min="25" max="25" width="11" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="8.375" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="28" width="7.375" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="16384" width="10.875" style="1"/>
+    <col min="26" max="26" width="8.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="28" width="7.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="29" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" ht="21" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="13"/>
@@ -3764,12 +3781,12 @@
       <c r="N1" s="13"/>
       <c r="O1" s="13"/>
     </row>
-    <row r="3" spans="1:26" ht="57" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:26" ht="57" x14ac:dyDescent="0.2">
       <c r="A3" s="19" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C3" s="20">
         <f>'Group and Self Assessment'!C10</f>
@@ -3858,15 +3875,15 @@
         <v>5</v>
       </c>
       <c r="Y3" s="21" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="Z3" s="12" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="4" spans="1:26" ht="144.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" ht="144.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="14" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B4" s="17">
         <v>0.1</v>
@@ -3877,7 +3894,9 @@
       <c r="D4" s="25">
         <v>0</v>
       </c>
-      <c r="E4" s="25"/>
+      <c r="E4" s="25">
+        <v>0</v>
+      </c>
       <c r="F4" s="25"/>
       <c r="G4" s="25"/>
       <c r="H4" s="25"/>
@@ -3892,32 +3911,32 @@
       <c r="Q4" s="25"/>
       <c r="R4" s="55">
         <f t="shared" ref="R4:R7" si="0">AVERAGE(C4:Q4)</f>
-        <v>2.5</v>
+        <v>1.6666666666666667</v>
       </c>
       <c r="S4" s="59" t="s">
+        <v>82</v>
+      </c>
+      <c r="T4" s="59" t="s">
         <v>83</v>
       </c>
-      <c r="T4" s="59" t="s">
+      <c r="U4" s="59" t="s">
         <v>84</v>
       </c>
-      <c r="U4" s="59" t="s">
+      <c r="V4" s="59" t="s">
         <v>85</v>
       </c>
-      <c r="V4" s="59" t="s">
+      <c r="W4" s="59" t="s">
         <v>86</v>
       </c>
-      <c r="W4" s="59" t="s">
+      <c r="X4" s="59" t="s">
         <v>87</v>
-      </c>
-      <c r="X4" s="59" t="s">
-        <v>88</v>
       </c>
       <c r="Y4" s="56"/>
       <c r="Z4" s="15"/>
     </row>
-    <row r="5" spans="1:26" ht="101.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:26" ht="101.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="14" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B5" s="17">
         <v>0.1</v>
@@ -3928,7 +3947,9 @@
       <c r="D5" s="25">
         <v>5</v>
       </c>
-      <c r="E5" s="25"/>
+      <c r="E5" s="25">
+        <v>5</v>
+      </c>
       <c r="F5" s="25"/>
       <c r="G5" s="25"/>
       <c r="H5" s="25"/>
@@ -3946,29 +3967,29 @@
         <v>5</v>
       </c>
       <c r="S5" s="59" t="s">
+        <v>89</v>
+      </c>
+      <c r="T5" s="59" t="s">
         <v>90</v>
       </c>
-      <c r="T5" s="59" t="s">
+      <c r="U5" s="59" t="s">
         <v>91</v>
       </c>
-      <c r="U5" s="59" t="s">
+      <c r="V5" s="59" t="s">
         <v>92</v>
       </c>
-      <c r="V5" s="59" t="s">
+      <c r="W5" s="59" t="s">
         <v>93</v>
       </c>
-      <c r="W5" s="59" t="s">
+      <c r="X5" s="59" t="s">
         <v>94</v>
-      </c>
-      <c r="X5" s="59" t="s">
-        <v>95</v>
       </c>
       <c r="Y5" s="56"/>
       <c r="Z5" s="15"/>
     </row>
-    <row r="6" spans="1:26" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:26" ht="51" x14ac:dyDescent="0.2">
       <c r="A6" s="14" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B6" s="17">
         <v>0.05</v>
@@ -3979,7 +4000,9 @@
       <c r="D6" s="25">
         <v>5</v>
       </c>
-      <c r="E6" s="25"/>
+      <c r="E6" s="25">
+        <v>5</v>
+      </c>
       <c r="F6" s="25"/>
       <c r="G6" s="25"/>
       <c r="H6" s="25"/>
@@ -3997,29 +4020,29 @@
         <v>5</v>
       </c>
       <c r="S6" s="59" t="s">
+        <v>96</v>
+      </c>
+      <c r="T6" s="59" t="s">
         <v>97</v>
       </c>
-      <c r="T6" s="59" t="s">
+      <c r="U6" s="59" t="s">
         <v>98</v>
       </c>
-      <c r="U6" s="59" t="s">
+      <c r="V6" s="59" t="s">
         <v>99</v>
       </c>
-      <c r="V6" s="59" t="s">
+      <c r="W6" s="59" t="s">
         <v>100</v>
       </c>
-      <c r="W6" s="59" t="s">
+      <c r="X6" s="59" t="s">
         <v>101</v>
-      </c>
-      <c r="X6" s="59" t="s">
-        <v>102</v>
       </c>
       <c r="Y6" s="56"/>
       <c r="Z6" s="15"/>
     </row>
-    <row r="7" spans="1:26" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:26" ht="51" x14ac:dyDescent="0.2">
       <c r="A7" s="14" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B7" s="17">
         <v>0.05</v>
@@ -4030,7 +4053,9 @@
       <c r="D7" s="25">
         <v>5</v>
       </c>
-      <c r="E7" s="25"/>
+      <c r="E7" s="25">
+        <v>5</v>
+      </c>
       <c r="F7" s="25"/>
       <c r="G7" s="25"/>
       <c r="H7" s="25"/>
@@ -4048,29 +4073,29 @@
         <v>5</v>
       </c>
       <c r="S7" s="59" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="T7" s="59" t="s">
+        <v>103</v>
+      </c>
+      <c r="U7" s="59" t="s">
         <v>104</v>
       </c>
-      <c r="U7" s="59" t="s">
+      <c r="V7" s="59" t="s">
         <v>105</v>
       </c>
-      <c r="V7" s="59" t="s">
+      <c r="W7" s="59" t="s">
         <v>106</v>
       </c>
-      <c r="W7" s="59" t="s">
+      <c r="X7" s="59" t="s">
         <v>107</v>
-      </c>
-      <c r="X7" s="59" t="s">
-        <v>108</v>
       </c>
       <c r="Y7" s="56"/>
       <c r="Z7" s="15"/>
     </row>
-    <row r="8" spans="1:26" ht="63" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:26" ht="68" x14ac:dyDescent="0.2">
       <c r="A8" s="14" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B8" s="17">
         <v>0.1</v>
@@ -4081,7 +4106,9 @@
       <c r="D8" s="25">
         <v>3</v>
       </c>
-      <c r="E8" s="25"/>
+      <c r="E8" s="25">
+        <v>3</v>
+      </c>
       <c r="F8" s="25"/>
       <c r="G8" s="25"/>
       <c r="H8" s="25"/>
@@ -4096,32 +4123,32 @@
       <c r="Q8" s="25"/>
       <c r="R8" s="55">
         <f t="shared" ref="R8:R12" si="1">AVERAGE(C8:Q8)</f>
-        <v>4</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="S8" s="59" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="T8" s="59" t="s">
+        <v>109</v>
+      </c>
+      <c r="U8" s="59" t="s">
         <v>110</v>
       </c>
-      <c r="U8" s="59" t="s">
+      <c r="V8" s="59" t="s">
         <v>111</v>
       </c>
-      <c r="V8" s="59" t="s">
+      <c r="W8" s="59" t="s">
         <v>112</v>
       </c>
-      <c r="W8" s="59" t="s">
+      <c r="X8" s="59" t="s">
         <v>113</v>
-      </c>
-      <c r="X8" s="59" t="s">
-        <v>114</v>
       </c>
       <c r="Y8" s="56"/>
       <c r="Z8" s="15"/>
     </row>
-    <row r="9" spans="1:26" ht="63" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:26" ht="68" x14ac:dyDescent="0.2">
       <c r="A9" s="14" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B9" s="17">
         <v>0.05</v>
@@ -4132,7 +4159,9 @@
       <c r="D9" s="25">
         <v>3</v>
       </c>
-      <c r="E9" s="25"/>
+      <c r="E9" s="25">
+        <v>4</v>
+      </c>
       <c r="F9" s="25"/>
       <c r="G9" s="25"/>
       <c r="H9" s="25"/>
@@ -4150,25 +4179,25 @@
         <v>4</v>
       </c>
       <c r="S9" s="59" t="s">
+        <v>115</v>
+      </c>
+      <c r="T9" s="59" t="s">
         <v>116</v>
-      </c>
-      <c r="T9" s="59" t="s">
-        <v>117</v>
       </c>
       <c r="U9" s="59"/>
       <c r="V9" s="59" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="W9" s="59"/>
       <c r="X9" s="59" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="Y9" s="56"/>
       <c r="Z9" s="15"/>
     </row>
-    <row r="10" spans="1:26" ht="78.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:26" ht="102" x14ac:dyDescent="0.2">
       <c r="A10" s="14" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B10" s="17">
         <v>0.1</v>
@@ -4179,7 +4208,9 @@
       <c r="D10" s="25">
         <v>0</v>
       </c>
-      <c r="E10" s="25"/>
+      <c r="E10" s="25">
+        <v>5</v>
+      </c>
       <c r="F10" s="25"/>
       <c r="G10" s="25"/>
       <c r="H10" s="25"/>
@@ -4194,32 +4225,32 @@
       <c r="Q10" s="25"/>
       <c r="R10" s="55">
         <f t="shared" si="2"/>
-        <v>2.5</v>
+        <v>3.3333333333333335</v>
       </c>
       <c r="S10" s="59" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="T10" s="59" t="s">
+        <v>120</v>
+      </c>
+      <c r="U10" s="59" t="s">
         <v>121</v>
       </c>
-      <c r="U10" s="59" t="s">
+      <c r="V10" s="59" t="s">
         <v>122</v>
       </c>
-      <c r="V10" s="59" t="s">
+      <c r="W10" s="59" t="s">
         <v>123</v>
       </c>
-      <c r="W10" s="59" t="s">
+      <c r="X10" s="59" t="s">
         <v>124</v>
-      </c>
-      <c r="X10" s="59" t="s">
-        <v>125</v>
       </c>
       <c r="Y10" s="56"/>
       <c r="Z10" s="15"/>
     </row>
-    <row r="11" spans="1:26" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:26" ht="34" x14ac:dyDescent="0.2">
       <c r="A11" s="14" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B11" s="17">
         <v>0.1</v>
@@ -4230,7 +4261,9 @@
       <c r="D11" s="25">
         <v>0</v>
       </c>
-      <c r="E11" s="25"/>
+      <c r="E11" s="25">
+        <v>5</v>
+      </c>
       <c r="F11" s="25"/>
       <c r="G11" s="25"/>
       <c r="H11" s="25"/>
@@ -4245,32 +4278,32 @@
       <c r="Q11" s="25"/>
       <c r="R11" s="55">
         <f t="shared" si="2"/>
-        <v>2.5</v>
+        <v>3.3333333333333335</v>
       </c>
       <c r="S11" s="59" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="T11" s="59" t="s">
+        <v>126</v>
+      </c>
+      <c r="U11" s="59" t="s">
         <v>127</v>
       </c>
-      <c r="U11" s="59" t="s">
+      <c r="V11" s="59" t="s">
         <v>128</v>
       </c>
-      <c r="V11" s="59" t="s">
+      <c r="W11" s="59" t="s">
         <v>129</v>
       </c>
-      <c r="W11" s="59" t="s">
+      <c r="X11" s="59" t="s">
         <v>130</v>
-      </c>
-      <c r="X11" s="59" t="s">
-        <v>131</v>
       </c>
       <c r="Y11" s="56"/>
       <c r="Z11" s="15"/>
     </row>
-    <row r="12" spans="1:26" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:26" ht="34" x14ac:dyDescent="0.2">
       <c r="A12" s="14" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B12" s="17">
         <v>0.1</v>
@@ -4281,7 +4314,9 @@
       <c r="D12" s="25">
         <v>0</v>
       </c>
-      <c r="E12" s="25"/>
+      <c r="E12" s="25">
+        <v>4</v>
+      </c>
       <c r="F12" s="25"/>
       <c r="G12" s="25"/>
       <c r="H12" s="25"/>
@@ -4296,32 +4331,32 @@
       <c r="Q12" s="25"/>
       <c r="R12" s="55">
         <f t="shared" si="1"/>
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="S12" s="59" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="T12" s="59" t="s">
+        <v>126</v>
+      </c>
+      <c r="U12" s="59" t="s">
         <v>127</v>
       </c>
-      <c r="U12" s="59" t="s">
+      <c r="V12" s="59" t="s">
         <v>128</v>
       </c>
-      <c r="V12" s="59" t="s">
+      <c r="W12" s="59" t="s">
         <v>129</v>
       </c>
-      <c r="W12" s="59" t="s">
+      <c r="X12" s="59" t="s">
         <v>130</v>
-      </c>
-      <c r="X12" s="59" t="s">
-        <v>131</v>
       </c>
       <c r="Y12" s="56"/>
       <c r="Z12" s="15"/>
     </row>
-    <row r="13" spans="1:26" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:26" ht="51" x14ac:dyDescent="0.2">
       <c r="A13" s="14" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B13" s="17">
         <v>0.1</v>
@@ -4332,7 +4367,9 @@
       <c r="D13" s="25">
         <v>5</v>
       </c>
-      <c r="E13" s="25"/>
+      <c r="E13" s="25">
+        <v>5</v>
+      </c>
       <c r="F13" s="25"/>
       <c r="G13" s="25"/>
       <c r="H13" s="25"/>
@@ -4350,29 +4387,29 @@
         <v>5</v>
       </c>
       <c r="S13" s="59" t="s">
+        <v>133</v>
+      </c>
+      <c r="T13" s="59" t="s">
         <v>134</v>
       </c>
-      <c r="T13" s="59" t="s">
+      <c r="U13" s="59" t="s">
         <v>135</v>
       </c>
-      <c r="U13" s="59" t="s">
+      <c r="V13" s="59" t="s">
         <v>136</v>
       </c>
-      <c r="V13" s="59" t="s">
+      <c r="W13" s="59" t="s">
         <v>137</v>
       </c>
-      <c r="W13" s="59" t="s">
+      <c r="X13" s="59" t="s">
         <v>138</v>
-      </c>
-      <c r="X13" s="59" t="s">
-        <v>139</v>
       </c>
       <c r="Y13" s="56"/>
       <c r="Z13" s="15"/>
     </row>
-    <row r="14" spans="1:26" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:26" ht="34" x14ac:dyDescent="0.2">
       <c r="A14" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B14" s="17">
         <v>0.15</v>
@@ -4383,7 +4420,9 @@
       <c r="D14" s="25">
         <v>5</v>
       </c>
-      <c r="E14" s="25"/>
+      <c r="E14" s="25">
+        <v>5</v>
+      </c>
       <c r="F14" s="25"/>
       <c r="G14" s="25"/>
       <c r="H14" s="25"/>
@@ -4401,29 +4440,29 @@
         <v>5</v>
       </c>
       <c r="S14" s="59" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="T14" s="59" t="s">
+        <v>126</v>
+      </c>
+      <c r="U14" s="59" t="s">
         <v>127</v>
       </c>
-      <c r="U14" s="59" t="s">
+      <c r="V14" s="59" t="s">
         <v>128</v>
       </c>
-      <c r="V14" s="59" t="s">
+      <c r="W14" s="59" t="s">
         <v>129</v>
       </c>
-      <c r="W14" s="59" t="s">
+      <c r="X14" s="59" t="s">
         <v>130</v>
-      </c>
-      <c r="X14" s="59" t="s">
-        <v>131</v>
       </c>
       <c r="Y14" s="56"/>
       <c r="Z14" s="15"/>
     </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:26" ht="17" x14ac:dyDescent="0.2">
       <c r="A15" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B15" s="18">
         <f>SUM(B4:B14)</f>
@@ -4439,7 +4478,7 @@
       </c>
       <c r="E15" s="7">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>4.1500000000000004</v>
       </c>
       <c r="F15" s="7">
         <f t="shared" si="4"/>
@@ -4499,9 +4538,9 @@
       <c r="Y15" s="7"/>
       <c r="Z15" s="15"/>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:26" ht="17" x14ac:dyDescent="0.2">
       <c r="A16" s="22" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B16" s="23"/>
       <c r="C16" s="23">
@@ -4514,7 +4553,7 @@
       </c>
       <c r="E16" s="23">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>16.600000000000001</v>
       </c>
       <c r="F16" s="23">
         <f t="shared" si="5"/>
@@ -4574,7 +4613,7 @@
       <c r="Y16" s="23"/>
       <c r="Z16" s="16"/>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" s="5"/>
     </row>
   </sheetData>
@@ -4589,21 +4628,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005836243B3C47804EAF5FFDD9F066FCC7" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9d21ddf3f0b128e39c9d770c8c903166">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b0326308c339679ad994635f2c691325" ns2:_="">
     <xsd:import namespace="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
@@ -4787,31 +4811,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D8D82CB-2E6F-4A14-B6B4-DFDD1BBD70FC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F61419B8-A98A-41CD-95EE-48A4F975B8D1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23B77F7C-EE47-4FBD-B078-6536C1487A1E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4827,4 +4842,28 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F61419B8-A98A-41CD-95EE-48A4F975B8D1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D8D82CB-2E6F-4A14-B6B4-DFDD1BBD70FC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>